<commit_message>
Enhance model output with timing summaries and improved data handling
</commit_message>
<xml_diff>
--- a/HanSong_Model/inputData.xlsx
+++ b/HanSong_Model/inputData.xlsx
@@ -1,22 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sillewiberg/Desktop/Skole/Speciale/Master-Thesis-eVTOL-1/HanSong_Model/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\HanSong_Model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E95AA517-A307-2B4E-89E5-0D548B37372A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A4BBC4-4F61-4437-9687-4475EE1D81D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="5860" windowWidth="28040" windowHeight="10920" activeTab="2" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="28800" windowHeight="15225" activeTab="4" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Infrastructure" sheetId="1" r:id="rId1"/>
     <sheet name="PassengerGroups" sheetId="2" r:id="rId2"/>
     <sheet name="PassengerGroups (2)" sheetId="3" r:id="rId3"/>
     <sheet name="Infrastructure (2)" sheetId="4" r:id="rId4"/>
+    <sheet name="Infrastructure (3)" sheetId="6" r:id="rId5"/>
+    <sheet name="PassengerGroups (3)" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="28">
   <si>
     <t>type</t>
   </si>
@@ -509,12 +511,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3245F359-CA05-2247-86C6-92433A84B0A2}">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="12.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -531,7 +533,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -551,7 +553,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -571,7 +573,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -591,7 +593,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -611,7 +613,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -639,9 +641,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0891C305-141D-384C-BB9E-30507F3FCDCC}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -661,7 +663,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -681,7 +683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -701,7 +703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -721,7 +723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -741,7 +743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -761,7 +763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -781,7 +783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -801,7 +803,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -821,7 +823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -841,7 +843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -869,9 +871,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF01B7F4-A8F2-E74F-93E1-1ACB4B99B891}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -891,7 +893,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -911,7 +913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -939,12 +941,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4154E97-9715-C248-8300-688A466787B4}">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="12.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -961,7 +963,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -981,7 +983,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1001,14 +1003,299 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I6" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30A04F2A-161E-4502-9547-1DD0A31CBA64}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="12.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E3CF6DF-5DC6-4F82-AD2C-07BC625FD2D9}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>25</v>
+      </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>50</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>70</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>40</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>110</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7">
+        <v>35</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>45</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Moved plane data to the input excel file
</commit_message>
<xml_diff>
--- a/HanSong_Model/inputData.xlsx
+++ b/HanSong_Model/inputData.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\HanSong_Model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A4BBC4-4F61-4437-9687-4475EE1D81D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C1D9AE8-356C-4FB3-A582-6B5BFF338217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="28800" windowHeight="15225" activeTab="4" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15225" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Infrastructure" sheetId="1" r:id="rId1"/>
-    <sheet name="PassengerGroups" sheetId="2" r:id="rId2"/>
-    <sheet name="PassengerGroups (2)" sheetId="3" r:id="rId3"/>
-    <sheet name="Infrastructure (2)" sheetId="4" r:id="rId4"/>
-    <sheet name="Infrastructure (3)" sheetId="6" r:id="rId5"/>
-    <sheet name="PassengerGroups (3)" sheetId="5" r:id="rId6"/>
+    <sheet name="PlaneData" sheetId="7" r:id="rId1"/>
+    <sheet name="Infrastructure" sheetId="1" r:id="rId2"/>
+    <sheet name="PassengerGroups" sheetId="2" r:id="rId3"/>
+    <sheet name="PassengerGroups (2)" sheetId="3" r:id="rId4"/>
+    <sheet name="Infrastructure (2)" sheetId="4" r:id="rId5"/>
+    <sheet name="Infrastructure (3)" sheetId="6" r:id="rId6"/>
+    <sheet name="PassengerGroups (3)" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="30">
   <si>
     <t>type</t>
   </si>
@@ -125,6 +126,12 @@
   </si>
   <si>
     <t>(37.4875, 127.1013)</t>
+  </si>
+  <si>
+    <t>Plane ID</t>
+  </si>
+  <si>
+    <t>Base Vertiport</t>
   </si>
 </sst>
 </file>
@@ -509,6 +516,59 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A94FE46B-0EE8-4D7E-956E-06AD6DDE4FF5}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3245F359-CA05-2247-86C6-92433A84B0A2}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -638,7 +698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0891C305-141D-384C-BB9E-30507F3FCDCC}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -868,7 +928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF01B7F4-A8F2-E74F-93E1-1ACB4B99B891}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -938,7 +998,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4154E97-9715-C248-8300-688A466787B4}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -1017,7 +1077,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30A04F2A-161E-4502-9547-1DD0A31CBA64}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -1132,7 +1192,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E3CF6DF-5DC6-4F82-AD2C-07BC625FD2D9}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Added progress printing when solving
</commit_message>
<xml_diff>
--- a/HanSong_Model/inputData.xlsx
+++ b/HanSong_Model/inputData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\HanSong_Model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C1D9AE8-356C-4FB3-A582-6B5BFF338217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F1877C7-F185-4351-8A8C-B51DCD0446C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15225" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="PlaneData" sheetId="7" r:id="rId1"/>
@@ -138,7 +138,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -157,6 +157,11 @@
       <color rgb="FF0A0A0A"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF000000"/>
+      <name val="CharisSIL"/>
     </font>
   </fonts>
   <fills count="2">
@@ -179,10 +184,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -700,7 +708,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0891C305-141D-384C-BB9E-30507F3FCDCC}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:X32"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -922,6 +930,320 @@
       <c r="F11">
         <v>1</v>
       </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>5</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12">
+        <v>30</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>20</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+      <c r="D14">
+        <v>50</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>4</v>
+      </c>
+      <c r="D15">
+        <v>35</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>16</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>4</v>
+      </c>
+      <c r="D16">
+        <v>20</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>17</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17">
+        <v>65</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>18</v>
+      </c>
+      <c r="B18">
+        <v>4</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18">
+        <v>90</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>19</v>
+      </c>
+      <c r="B19">
+        <v>5</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
+        <v>15</v>
+      </c>
+      <c r="E19">
+        <v>2</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>20</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="C20">
+        <v>4</v>
+      </c>
+      <c r="D20">
+        <v>60</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="Q23" s="3"/>
+      <c r="R23" s="3"/>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+      <c r="P24" s="3"/>
+      <c r="Q24" s="3"/>
+      <c r="R24" s="3"/>
+      <c r="S24" s="3"/>
+      <c r="T24" s="3"/>
+      <c r="U24" s="3"/>
+      <c r="V24" s="3"/>
+      <c r="W24" s="3"/>
+      <c r="X24" s="3"/>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="3"/>
+      <c r="V25" s="3"/>
+      <c r="W25" s="3"/>
+      <c r="X25" s="3"/>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+      <c r="P26" s="3"/>
+      <c r="Q26" s="3"/>
+      <c r="R26" s="3"/>
+      <c r="S26" s="3"/>
+      <c r="T26" s="3"/>
+      <c r="U26" s="3"/>
+      <c r="V26" s="3"/>
+      <c r="W26" s="3"/>
+      <c r="X26" s="3"/>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+      <c r="R27" s="3"/>
+      <c r="S27" s="3"/>
+      <c r="T27" s="3"/>
+      <c r="U27" s="3"/>
+      <c r="V27" s="3"/>
+      <c r="W27" s="3"/>
+      <c r="X27" s="3"/>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="3"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
+      <c r="U28" s="3"/>
+      <c r="V28" s="3"/>
+      <c r="W28" s="3"/>
+      <c r="X28" s="3"/>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3"/>
+      <c r="R29" s="3"/>
+      <c r="S29" s="3"/>
+      <c r="T29" s="3"/>
+      <c r="U29" s="3"/>
+      <c r="V29" s="3"/>
+      <c r="W29" s="3"/>
+      <c r="X29" s="3"/>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+      <c r="P30" s="3"/>
+      <c r="Q30" s="3"/>
+      <c r="R30" s="3"/>
+      <c r="S30" s="3"/>
+      <c r="T30" s="3"/>
+      <c r="U30" s="3"/>
+      <c r="V30" s="3"/>
+      <c r="W30" s="3"/>
+      <c r="X30" s="3"/>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M31" s="3"/>
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+      <c r="P31" s="3"/>
+      <c r="Q31" s="3"/>
+      <c r="R31" s="3"/>
+      <c r="S31" s="3"/>
+      <c r="T31" s="3"/>
+      <c r="U31" s="3"/>
+      <c r="V31" s="3"/>
+      <c r="W31" s="3"/>
+      <c r="X31" s="3"/>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M32" s="3"/>
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
+      <c r="P32" s="3"/>
+      <c r="Q32" s="3"/>
+      <c r="R32" s="3"/>
+      <c r="S32" s="3"/>
+      <c r="T32" s="3"/>
+      <c r="U32" s="3"/>
+      <c r="V32" s="3"/>
+      <c r="W32" s="3"/>
+      <c r="X32" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Refactor code structure for improved readability a nd maintainability
</commit_message>
<xml_diff>
--- a/HanSong_Model/inputData.xlsx
+++ b/HanSong_Model/inputData.xlsx
@@ -1,29 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sillewiberg/Desktop/Skole/Speciale/Master-Thesis-eVTOL-1/HanSong_Model/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/asbb/Desktop/Speciale/Master-Thesis-eVTOL/HanSong_Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7473B2F8-CE9E-DC40-B158-DDACBE492212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7816C04-DD99-0F4D-9593-D4905A02CF31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="10000" windowHeight="16340" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="16560" windowHeight="18380" activeTab="3" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Parameters" sheetId="9" r:id="rId1"/>
-    <sheet name="PlaneData" sheetId="7" r:id="rId2"/>
-    <sheet name="PlaneData (2)" sheetId="8" r:id="rId3"/>
-    <sheet name="Infrastructure" sheetId="1" r:id="rId4"/>
-    <sheet name="PassengerGroups" sheetId="2" r:id="rId5"/>
-    <sheet name="PassengerGroups (2)" sheetId="3" r:id="rId6"/>
-    <sheet name="Infrastructure (2)" sheetId="4" r:id="rId7"/>
-    <sheet name="Infrastructure (3)" sheetId="6" r:id="rId8"/>
-    <sheet name="PassengerGroups (3)" sheetId="5" r:id="rId9"/>
+    <sheet name="PlaneData" sheetId="7" r:id="rId1"/>
+    <sheet name="PlaneData (2)" sheetId="8" r:id="rId2"/>
+    <sheet name="Infrastructure" sheetId="1" r:id="rId3"/>
+    <sheet name="PassengerGroups" sheetId="2" r:id="rId4"/>
+    <sheet name="PassengerGroups (2)" sheetId="3" r:id="rId5"/>
+    <sheet name="Infrastructure (2)" sheetId="4" r:id="rId6"/>
+    <sheet name="Infrastructure (3)" sheetId="6" r:id="rId7"/>
+    <sheet name="PassengerGroups (3)" sheetId="5" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="30">
   <si>
     <t>type</t>
   </si>
@@ -52,6 +51,9 @@
     <t>vertiport</t>
   </si>
   <si>
+    <t>vertistop</t>
+  </si>
+  <si>
     <t>id</t>
   </si>
   <si>
@@ -131,94 +133,13 @@
   </si>
   <si>
     <t>Base Vertiport</t>
-  </si>
-  <si>
-    <t>cap_flt</t>
-  </si>
-  <si>
-    <t>cap_u</t>
-  </si>
-  <si>
-    <t>bmax</t>
-  </si>
-  <si>
-    <t>bmin</t>
-  </si>
-  <si>
-    <t>ec</t>
-  </si>
-  <si>
-    <t>te</t>
-  </si>
-  <si>
-    <t>w</t>
-  </si>
-  <si>
-    <t>ET</t>
-  </si>
-  <si>
-    <t>fd_{i,j} = $3/km</t>
-  </si>
-  <si>
-    <t>fs_{i,j}=75% of fd_{i,j}</t>
-  </si>
-  <si>
-    <t>p_a = $10</t>
-  </si>
-  <si>
-    <t>c_{i,j} = $1/km</t>
-  </si>
-  <si>
-    <t>e_{i,j} = 1%/km</t>
-  </si>
-  <si>
-    <t>rt_{i,j} = 0.6 min/km</t>
-  </si>
-  <si>
-    <t>capacity of air corridor</t>
-  </si>
-  <si>
-    <t>seat capacity of eVTOL</t>
-  </si>
-  <si>
-    <t>5% battery charged per unit time</t>
-  </si>
-  <si>
-    <t>minimum turnaround time at vertiport</t>
-  </si>
-  <si>
-    <t>maximum waiting time</t>
-  </si>
-  <si>
-    <t>end time</t>
-  </si>
-  <si>
-    <t>fare_stopover_factor</t>
-  </si>
-  <si>
-    <t>p_penalty</t>
-  </si>
-  <si>
-    <t>operating_cost_per_km</t>
-  </si>
-  <si>
-    <t>battery_per_km</t>
-  </si>
-  <si>
-    <t>time_per_km</t>
-  </si>
-  <si>
-    <t>fare_direct_per_km</t>
-  </si>
-  <si>
-    <t>Parameters</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -243,6 +164,13 @@
       <color rgb="FF000000"/>
       <name val="CharisSIL"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -264,15 +192,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -606,179 +533,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B15C49E0-A7B4-734A-8962-DC2A879F4079}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <cols>
-    <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" style="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="5">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="5">
-        <v>0.75</v>
-      </c>
-      <c r="D3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5">
-        <v>10</v>
-      </c>
-      <c r="D4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B5" s="5">
-        <v>1.51</v>
-      </c>
-      <c r="D5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" s="5">
-        <v>0.3</v>
-      </c>
-      <c r="D6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" s="5">
-        <v>0.2</v>
-      </c>
-      <c r="D7" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="5">
-        <v>1</v>
-      </c>
-      <c r="D8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="5">
-        <v>4</v>
-      </c>
-      <c r="D9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="5">
-        <v>100</v>
-      </c>
-      <c r="D10" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="5">
-        <v>10</v>
-      </c>
-      <c r="D11" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="5">
-        <v>5</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="5">
-        <v>10</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="5">
-        <v>10</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="5">
-        <v>240</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A94FE46B-0EE8-4D7E-956E-06AD6DDE4FF5}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
@@ -788,10 +542,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -831,8 +585,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A48C4B-C23A-0343-9CD4-B20C0FE9227B}">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C31D2D17-FC72-FE49-9329-D197D3094A2B}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
@@ -841,10 +595,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -860,7 +614,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -868,7 +622,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3245F359-CA05-2247-86C6-92433A84B0A2}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
@@ -881,16 +635,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -904,13 +658,13 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -924,18 +678,18 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -944,18 +698,18 @@
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -964,18 +718,18 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -984,13 +738,13 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -998,33 +752,29 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0891C305-141D-384C-BB9E-30507F3FCDCC}">
   <dimension ref="A1:X32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
-  <cols>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="11.5" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1111,11 +861,11 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
+      <c r="B6" s="4">
+        <v>2</v>
+      </c>
+      <c r="C6" s="4">
+        <v>3</v>
       </c>
       <c r="D6">
         <v>110</v>
@@ -1151,11 +901,11 @@
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8">
-        <v>3</v>
+      <c r="B8" s="4">
+        <v>5</v>
+      </c>
+      <c r="C8" s="4">
+        <v>1</v>
       </c>
       <c r="D8">
         <v>45</v>
@@ -1171,11 +921,11 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9">
-        <v>2</v>
-      </c>
-      <c r="C9">
-        <v>3</v>
+      <c r="B9" s="4">
+        <v>3</v>
+      </c>
+      <c r="C9" s="4">
+        <v>2</v>
       </c>
       <c r="D9">
         <v>60</v>
@@ -1191,11 +941,11 @@
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10">
-        <v>2</v>
-      </c>
-      <c r="C10">
-        <v>3</v>
+      <c r="B10" s="4">
+        <v>5</v>
+      </c>
+      <c r="C10" s="4">
+        <v>2</v>
       </c>
       <c r="D10">
         <v>40</v>
@@ -1251,11 +1001,11 @@
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="4">
+        <v>2</v>
+      </c>
+      <c r="C13" s="4">
         <v>5</v>
-      </c>
-      <c r="C13">
-        <v>2</v>
       </c>
       <c r="D13">
         <v>30</v>
@@ -1351,11 +1101,11 @@
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18">
-        <v>3</v>
-      </c>
-      <c r="C18">
-        <v>2</v>
+      <c r="B18" s="4">
+        <v>2</v>
+      </c>
+      <c r="C18" s="4">
+        <v>3</v>
       </c>
       <c r="D18">
         <v>65</v>
@@ -1371,11 +1121,11 @@
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="4">
+        <v>3</v>
+      </c>
+      <c r="C19" s="4">
         <v>4</v>
-      </c>
-      <c r="C19">
-        <v>2</v>
       </c>
       <c r="D19">
         <v>90</v>
@@ -1411,11 +1161,11 @@
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21">
-        <v>3</v>
-      </c>
-      <c r="C21">
-        <v>4</v>
+      <c r="B21" s="4">
+        <v>1</v>
+      </c>
+      <c r="C21" s="4">
+        <v>3</v>
       </c>
       <c r="D21">
         <v>60</v>
@@ -1566,29 +1316,29 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF01B7F4-A8F2-E74F-93E1-1ACB4B99B891}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1636,7 +1386,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4154E97-9715-C248-8300-688A466787B4}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
@@ -1649,16 +1399,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -1672,13 +1422,13 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1692,13 +1442,13 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1708,6 +1458,121 @@
       <c r="I5" s="1"/>
     </row>
     <row r="6" spans="1:11">
+      <c r="I6" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30A04F2A-161E-4502-9547-1DD0A31CBA64}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <cols>
+    <col min="3" max="3" width="12.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
       <c r="I6" s="1"/>
     </row>
   </sheetData>
@@ -1716,161 +1581,28 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30A04F2A-161E-4502-9547-1DD0A31CBA64}">
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
-  <cols>
-    <col min="3" max="3" width="12.6640625" customWidth="1"/>
-    <col min="4" max="4" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.5" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E3CF6DF-5DC6-4F82-AD2C-07BC625FD2D9}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:6">

</xml_diff>

<commit_message>
Update inputData.xlsx with new data
</commit_message>
<xml_diff>
--- a/HanSong_Model/inputData.xlsx
+++ b/HanSong_Model/inputData.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65564938-94FB-44AE-953A-A74912A52C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="9" r:id="rId1"/>
@@ -2081,7 +2081,7 @@
       </c>
       <c r="D2">
         <f ca="1">RANDBETWEEN(10,120)</f>
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -2091,11 +2091,11 @@
       </c>
       <c r="I2">
         <f ca="1">RANDBETWEEN(1,5)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <f ca="1">RANDBETWEEN(1,5)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L2">
         <f ca="1">RANDBETWEEN(1,5)</f>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="D3">
         <f t="shared" ref="D3:D21" ca="1" si="0">RANDBETWEEN(10,120)</f>
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -2124,15 +2124,15 @@
       </c>
       <c r="I3">
         <f t="shared" ref="I3:I21" ca="1" si="1">RANDBETWEEN(1,5)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K3">
         <f t="shared" ref="K3:L21" ca="1" si="2">RANDBETWEEN(1,5)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L3">
         <f t="shared" ca="1" si="2"/>
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="D4">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>57</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -2157,15 +2157,15 @@
       </c>
       <c r="I4">
         <f t="shared" ca="1" si="1"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K4">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L4">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="D5">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>67</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -2190,11 +2190,11 @@
       </c>
       <c r="I5">
         <f t="shared" ca="1" si="1"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K5">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L5">
         <f t="shared" ca="1" si="2"/>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="D6">
         <f t="shared" ca="1" si="0"/>
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2223,15 +2223,15 @@
       </c>
       <c r="I6">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6">
         <f t="shared" ca="1" si="2"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L6">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="D7">
         <f t="shared" ca="1" si="0"/>
-        <v>42</v>
+        <v>104</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2256,15 +2256,15 @@
       </c>
       <c r="I7">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K7">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L7">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="D8">
         <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2289,15 +2289,15 @@
       </c>
       <c r="I8">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K8">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L8">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="D9">
         <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <v>48</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="I9">
         <f t="shared" ca="1" si="1"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K9">
         <f t="shared" ca="1" si="2"/>
@@ -2330,7 +2330,7 @@
       </c>
       <c r="L9">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D10">
         <f t="shared" ca="1" si="0"/>
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -2355,15 +2355,15 @@
       </c>
       <c r="I10">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L10">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="D11">
         <f t="shared" ca="1" si="0"/>
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2388,11 +2388,11 @@
       </c>
       <c r="I11">
         <f t="shared" ca="1" si="1"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K11">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L11">
         <f t="shared" ca="1" si="2"/>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="D12">
         <f t="shared" ca="1" si="0"/>
-        <v>18</v>
+        <v>92</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2425,11 +2425,11 @@
       </c>
       <c r="K12">
         <f t="shared" ca="1" si="2"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L12">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="D13">
         <f t="shared" ca="1" si="0"/>
-        <v>15</v>
+        <v>115</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -2454,11 +2454,11 @@
       </c>
       <c r="I13">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L13">
         <f t="shared" ca="1" si="2"/>
@@ -2477,7 +2477,7 @@
       </c>
       <c r="D14">
         <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <v>24</v>
       </c>
       <c r="E14">
         <v>2</v>
@@ -2487,15 +2487,15 @@
       </c>
       <c r="I14">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14">
         <f t="shared" ca="1" si="2"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L14">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="D15">
         <f t="shared" ca="1" si="0"/>
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="I15">
         <f t="shared" ca="1" si="1"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K15">
         <f t="shared" ca="1" si="2"/>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="D16">
         <f t="shared" ca="1" si="0"/>
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="E16">
         <v>3</v>
@@ -2553,15 +2553,15 @@
       </c>
       <c r="I16">
         <f t="shared" ca="1" si="1"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K16">
         <f t="shared" ca="1" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="L16">
+        <f t="shared" ca="1" si="2"/>
         <v>5</v>
-      </c>
-      <c r="L16">
-        <f t="shared" ca="1" si="2"/>
-        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:24">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="D17">
         <f t="shared" ca="1" si="0"/>
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="E17">
         <v>3</v>
@@ -2586,15 +2586,15 @@
       </c>
       <c r="I17">
         <f t="shared" ca="1" si="1"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K17">
         <f t="shared" ca="1" si="2"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L17">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:24">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="D18">
         <f t="shared" ca="1" si="0"/>
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="E18">
         <v>2</v>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="I18">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K18">
         <f t="shared" ca="1" si="2"/>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="L18">
         <f t="shared" ca="1" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:24">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="D19">
         <f t="shared" ca="1" si="0"/>
-        <v>67</v>
+        <v>24</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -2652,15 +2652,15 @@
       </c>
       <c r="I19">
         <f t="shared" ca="1" si="1"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K19">
         <f t="shared" ca="1" si="2"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:24">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="D20">
         <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="E20">
         <v>2</v>
@@ -2685,11 +2685,11 @@
       </c>
       <c r="I20">
         <f t="shared" ca="1" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L20">
         <f t="shared" ca="1" si="2"/>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="D21">
         <f t="shared" ca="1" si="0"/>
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="K21">
         <f t="shared" ca="1" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L21">
         <f t="shared" ca="1" si="2"/>

</xml_diff>